<commit_message>
Day06 Project Update with Readme
</commit_message>
<xml_diff>
--- a/sales_data.xlsx
+++ b/sales_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python-Freelancing\Day06-Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3341F470-93F1-4D36-9F1D-817F6F794F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC200A7-65EF-4490-A03F-067FE10F88ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -461,7 +461,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="2">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>